<commit_message>
:bat: excel table with 16S and ITS CCA results
</commit_message>
<xml_diff>
--- a/plots/5_LBM&co/combined cca results.xlsx
+++ b/plots/5_LBM&co/combined cca results.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="12">
   <si>
     <t/>
   </si>
@@ -63,7 +63,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="2">
     <numFmt numFmtId="164" formatCode="0.0"/>
-    <numFmt numFmtId="169" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -94,15 +94,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -400,25 +403,30 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F7"/>
+  <dimension ref="A1:H7"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="30" bestFit="1" customWidth="1"/>
     <col min="5" max="6" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="19.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="C1" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
@@ -431,11 +439,17 @@
       <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="H2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B3" s="4" t="s">
         <v>5</v>
       </c>
@@ -448,11 +462,17 @@
       <c r="E3" s="1">
         <v>0.8</v>
       </c>
-      <c r="F3">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F3" s="2">
+        <v>1.2473676861168901</v>
+      </c>
+      <c r="G3" s="2">
+        <v>10.4803218548867</v>
+      </c>
+      <c r="H3">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
@@ -465,11 +485,17 @@
       <c r="E4" s="1">
         <v>0.1</v>
       </c>
-      <c r="F4">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F4" s="2">
+        <v>0.61800168827312596</v>
+      </c>
+      <c r="G4" s="2">
+        <v>2.8082190067316399</v>
+      </c>
+      <c r="H4">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B5" s="4" t="s">
         <v>7</v>
       </c>
@@ -482,11 +508,17 @@
       <c r="E5" s="1">
         <v>0.1</v>
       </c>
-      <c r="F5">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F5" s="2">
+        <v>1.86205011672485</v>
+      </c>
+      <c r="G5" s="2">
+        <v>6.5687013560600196</v>
+      </c>
+      <c r="H5">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B6" s="4" t="s">
         <v>8</v>
       </c>
@@ -499,11 +531,17 @@
       <c r="E6" s="1">
         <v>0.1</v>
       </c>
-      <c r="F6">
-        <v>0.1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F6" s="2">
+        <v>1.2440484284517199</v>
+      </c>
+      <c r="G6" s="2">
+        <v>11.2993693295311</v>
+      </c>
+      <c r="H6">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="B7" s="4" t="s">
         <v>9</v>
       </c>
@@ -516,11 +554,21 @@
       <c r="E7" s="1">
         <v>0.1</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="2">
+        <v>0.61468243060795802</v>
+      </c>
+      <c r="G7" s="2">
+        <v>3.3976549841584198</v>
+      </c>
+      <c r="H7">
         <v>0.1</v>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="F1:H1"/>
+    <mergeCell ref="C1:E1"/>
+  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>